<commit_message>
Mejora agregar el numero de operador a la plantilla de Whatsapp
</commit_message>
<xml_diff>
--- a/historial de versiones/historial de versiones.xlsx
+++ b/historial de versiones/historial de versiones.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ReneGonzalez\nglobal_donpedro\historial de versiones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D0E4D43-32F5-4846-A49E-25DB8369FC25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B71EEAF0-12A7-4AE7-9C5F-0C2FD928C5E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28908" yWindow="-108" windowWidth="29016" windowHeight="15696" xr2:uid="{D8516950-B82A-44A6-A6D8-9588F2ED2E08}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>CONTROL DE VERSIONES APP DON PEDRO</t>
   </si>
@@ -144,6 +144,12 @@
   </si>
   <si>
     <t>Mejora para que solamente envié mensaje de alerta cuando el estatus es diferente a: Finalizado, Cancelado, Hold FDA y Review FDA.</t>
+  </si>
+  <si>
+    <t>1.7.1</t>
+  </si>
+  <si>
+    <t>Mejora para que en los campos de Temperatura Mínima y Máxima, las tome de la tabla de productos desde la BD, en caso de tener mas de 1 producto, promedia los valores, adicional queda habilitado para editar los valores</t>
   </si>
 </sst>
 </file>
@@ -207,11 +213,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -225,7 +228,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -560,153 +565,160 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36194886-2769-4A79-9B82-6C17CD89E475}">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="70.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="B1" s="6"/>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
+    <row r="10" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
+    <row r="12" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F12" s="7"/>
-    </row>
-    <row r="13" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
+    </row>
+    <row r="13" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="4" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="4" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mejora exportar historial a de despachos a excel y que mande el numero de celular en las alertas
</commit_message>
<xml_diff>
--- a/historial de versiones/historial de versiones.xlsx
+++ b/historial de versiones/historial de versiones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ReneGonzalez\nglobal_donpedro\historial de versiones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B71EEAF0-12A7-4AE7-9C5F-0C2FD928C5E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45FFAE3B-5DAF-4483-B168-4E53374B164C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28908" yWindow="-108" windowWidth="29016" windowHeight="15696" xr2:uid="{D8516950-B82A-44A6-A6D8-9588F2ED2E08}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D8516950-B82A-44A6-A6D8-9588F2ED2E08}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>CONTROL DE VERSIONES APP DON PEDRO</t>
   </si>
@@ -150,6 +150,18 @@
   </si>
   <si>
     <t>Mejora para que en los campos de Temperatura Mínima y Máxima, las tome de la tabla de productos desde la BD, en caso de tener mas de 1 producto, promedia los valores, adicional queda habilitado para editar los valores</t>
+  </si>
+  <si>
+    <t>1.7.2</t>
+  </si>
+  <si>
+    <t>Mejora para que en el grid de Operaciones USA, solamente muestre los datos del año en curso</t>
+  </si>
+  <si>
+    <t>1.7.3</t>
+  </si>
+  <si>
+    <t>Mejora para exportar en un rango de fecha los despachos finalizados a excel, sin importar de que año sea.</t>
   </si>
 </sst>
 </file>
@@ -565,7 +577,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36194886-2769-4A79-9B82-6C17CD89E475}">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="70.77734375" bestFit="1" customWidth="1"/>
@@ -721,6 +733,22 @@
         <v>36</v>
       </c>
     </row>
+    <row r="21" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
Mejora prorrateo de costo por caja
</commit_message>
<xml_diff>
--- a/historial de versiones/historial de versiones.xlsx
+++ b/historial de versiones/historial de versiones.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ReneGonzalez\nglobal_donpedro\historial de versiones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45FFAE3B-5DAF-4483-B168-4E53374B164C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA0E50B3-41CA-45BE-873C-F76810E5F719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D8516950-B82A-44A6-A6D8-9588F2ED2E08}"/>
+    <workbookView xWindow="-28908" yWindow="-108" windowWidth="29016" windowHeight="15696" xr2:uid="{D8516950-B82A-44A6-A6D8-9588F2ED2E08}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t>CONTROL DE VERSIONES APP DON PEDRO</t>
   </si>
@@ -162,6 +163,42 @@
   </si>
   <si>
     <t>Mejora para exportar en un rango de fecha los despachos finalizados a excel, sin importar de que año sea.</t>
+  </si>
+  <si>
+    <t>1.7.4</t>
+  </si>
+  <si>
+    <t>Mejora, se agrega el numero de celular de Whatsapp del operador en los mensajes de alerta por Whatsapp</t>
+  </si>
+  <si>
+    <t>1.7.5</t>
+  </si>
+  <si>
+    <t>Mejora para agregar un despacho nuevo sin crear programacion lider.</t>
+  </si>
+  <si>
+    <t>1.7.6</t>
+  </si>
+  <si>
+    <t>Mejora agregar select dinamico en Proyecto al crear nuevo despacho sin Programacion del lider.</t>
+  </si>
+  <si>
+    <t>1.7.7</t>
+  </si>
+  <si>
+    <t>Agregar cargos extras al flete desde el boton de incidencias.</t>
+  </si>
+  <si>
+    <t>1.7.8</t>
+  </si>
+  <si>
+    <t>En control de pagos, al liquidar un flete, el monto del flete que se captura en el despacho lo agrega al campo monto flete y en comentarios cargos extras enlista los cargos capturados, tambien se habilita la carga de PDF de la factura</t>
+  </si>
+  <si>
+    <t>1.7.9</t>
+  </si>
+  <si>
+    <t>Se corrigio los viajes consolidados al crear un nuevo despacho con varias programaciones del lider. Ahora se puede seleccionar varias programaciones del lider o varios proyectos sin que haya programacion del lider</t>
   </si>
 </sst>
 </file>
@@ -258,6 +295,1243 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>83820</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>449580</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>168480</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="Rectángulo: esquinas redondeadas 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7D2D3EBE-421D-05F7-60F7-20EF24362D68}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="83820" y="182880"/>
+          <a:ext cx="2743200" cy="900000"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>375838</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2131033" cy="953466"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="CuadroTexto 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8E88A00D-F977-1F64-6B52-45D5B42B5D89}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="375838" y="182880"/>
+          <a:ext cx="2131033" cy="953466"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>CHILE CHILTEPÍN DESHIDRATADO</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>CALIDAD: L</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>Cont.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100" baseline="0"/>
+            <a:t> Neto: 100 gr</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100" baseline="0"/>
+            <a:t>**Productos sin etiqueta**</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>373380</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>840</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="Rectángulo: esquinas redondeadas 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EEBE9EDF-E682-471B-82EC-9719F6DAA02C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3177540" y="198120"/>
+          <a:ext cx="2743200" cy="900000"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>299638</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2131033" cy="953466"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="CuadroTexto 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B826FF27-ED59-437C-A00C-E53F065F9536}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3469558" y="198120"/>
+          <a:ext cx="2131033" cy="953466"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>CHILE CHILTEPÍN DESHIDRATADO</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>CALIDAD: L</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>Cont.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100" baseline="0"/>
+            <a:t> Neto: 100 gr</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100" baseline="0"/>
+            <a:t>**Productos sin etiqueta**</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>83820</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>449580</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>46560</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="Rectángulo: esquinas redondeadas 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{001F406E-5006-4473-A39B-0A63384239A7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="83820" y="1341120"/>
+          <a:ext cx="2743200" cy="900000"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>375838</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2131033" cy="953466"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="CuadroTexto 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{16172630-1E01-48D6-AA4E-AE99903AC75A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="375838" y="1341120"/>
+          <a:ext cx="2131033" cy="953466"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>CHILE CHILTEPÍN DESHIDRATADO</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>CALIDAD: L</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>Cont.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100" baseline="0"/>
+            <a:t> Neto: 100 gr</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100" baseline="0"/>
+            <a:t>**Productos sin etiqueta**</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>373380</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>61800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="Rectángulo: esquinas redondeadas 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AABABD8F-077D-4D5C-8ADA-27A5B8EA433F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3177540" y="1356360"/>
+          <a:ext cx="2743200" cy="900000"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>299638</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2131033" cy="953466"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="CuadroTexto 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3879AC06-3ED3-4225-B9DC-B9304FEC8E88}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3469558" y="1356360"/>
+          <a:ext cx="2131033" cy="953466"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>CHILE CHILTEPÍN DESHIDRATADO</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>CALIDAD: L</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>Cont.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100" baseline="0"/>
+            <a:t> Neto: 100 gr</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100" baseline="0"/>
+            <a:t>**Productos sin etiqueta**</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>434340</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>145620</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="Rectángulo: esquinas redondeadas 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{86808AAA-E903-4A50-9555-999981048455}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="68580" y="2537460"/>
+          <a:ext cx="2743200" cy="900000"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>360598</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2131033" cy="953466"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="CuadroTexto 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{11B919BD-DD0D-4E33-822E-C52083758CFE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="360598" y="2537460"/>
+          <a:ext cx="2131033" cy="953466"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>CHILE CHILTEPÍN DESHIDRATADO</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>CALIDAD: L</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>Cont.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100" baseline="0"/>
+            <a:t> Neto: 100 gr</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100" baseline="0"/>
+            <a:t>**Productos sin etiqueta**</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>784860</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>358140</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>160860</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="12" name="Rectángulo: esquinas redondeadas 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{188CF810-7F78-42C7-BE9F-C7C7FA06A176}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3162300" y="2552700"/>
+          <a:ext cx="2743200" cy="900000"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>284398</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2131033" cy="953466"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13" name="CuadroTexto 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{596BD488-0CAD-42C1-A4FB-3552C34AA228}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3454318" y="2552700"/>
+          <a:ext cx="2131033" cy="953466"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>CHILE CHILTEPÍN DESHIDRATADO</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>CALIDAD: L</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>Cont.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100" baseline="0"/>
+            <a:t> Neto: 100 gr</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100" baseline="0"/>
+            <a:t>**Productos sin etiqueta**</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>434340</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>8460</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="14" name="Rectángulo: esquinas redondeadas 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3250C282-DFC0-4E14-9A4F-90832BA09322}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="68580" y="3680460"/>
+          <a:ext cx="2743200" cy="900000"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>360598</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2131033" cy="953466"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="CuadroTexto 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DACFD36E-9611-4930-9EEF-011EF9E92E78}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="360598" y="3680460"/>
+          <a:ext cx="2131033" cy="953466"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>CHILE CHILTEPÍN DESHIDRATADO</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>CALIDAD: L</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>Cont.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100" baseline="0"/>
+            <a:t> Neto: 100 gr</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100" baseline="0"/>
+            <a:t>**Productos sin etiqueta**</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>784860</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>358140</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>23700</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="16" name="Rectángulo: esquinas redondeadas 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ECFBEBF8-49C5-4E33-91D1-8A03A2549406}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3162300" y="3695700"/>
+          <a:ext cx="2743200" cy="900000"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>284398</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2131033" cy="953466"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="17" name="CuadroTexto 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ED9DCBC7-28F5-4338-A6F9-7EED00F21F80}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3454318" y="3695700"/>
+          <a:ext cx="2131033" cy="953466"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>CHILE CHILTEPÍN DESHIDRATADO</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>CALIDAD: L</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100"/>
+            <a:t>Cont.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100" baseline="0"/>
+            <a:t> Neto: 100 gr</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-MX" sz="1100" baseline="0"/>
+            <a:t>**Productos sin etiqueta**</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="es-MX" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -577,7 +1851,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36194886-2769-4A79-9B82-6C17CD89E475}">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="70.77734375" bestFit="1" customWidth="1"/>
@@ -749,10 +2023,69 @@
         <v>40</v>
       </c>
     </row>
+    <row r="23" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B42FC5CD-2AD4-4076-ACC2-3159794E5CE4}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Mejora control de pagos
</commit_message>
<xml_diff>
--- a/historial de versiones/historial de versiones.xlsx
+++ b/historial de versiones/historial de versiones.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ReneGonzalez\nglobal_donpedro\historial de versiones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA0E50B3-41CA-45BE-873C-F76810E5F719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08113729-0247-4026-BE02-0021DA82B126}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28908" yWindow="-108" windowWidth="29016" windowHeight="15696" xr2:uid="{D8516950-B82A-44A6-A6D8-9588F2ED2E08}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D8516950-B82A-44A6-A6D8-9588F2ED2E08}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
   <si>
     <t>CONTROL DE VERSIONES APP DON PEDRO</t>
   </si>
@@ -199,6 +199,54 @@
   </si>
   <si>
     <t>Se corrigio los viajes consolidados al crear un nuevo despacho con varias programaciones del lider. Ahora se puede seleccionar varias programaciones del lider o varios proyectos sin que haya programacion del lider</t>
+  </si>
+  <si>
+    <t>1.8.0</t>
+  </si>
+  <si>
+    <t>Mejora control de pagos, el formato de moneda se configura a Pesos MXN.</t>
+  </si>
+  <si>
+    <t>1.8.1</t>
+  </si>
+  <si>
+    <t>Mejora el monto capturado del flete en despacho lo muestra en costo flete base.</t>
+  </si>
+  <si>
+    <t>1.8.2</t>
+  </si>
+  <si>
+    <t>En el cuadro de comentarios e incidencias muestra un desgloce de cargos extras capturados en Operaciones USA</t>
+  </si>
+  <si>
+    <t>1.8.3</t>
+  </si>
+  <si>
+    <t>Mejora, se agrega prorrateo de multi clientes, se selecciona el cliente por producto.</t>
+  </si>
+  <si>
+    <t>1.8.4</t>
+  </si>
+  <si>
+    <t>Se habilita la carga PDF de la factura</t>
+  </si>
+  <si>
+    <t>1.8.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se agrega "Requiere servicios complementarios" para que aparezca el id de viaje en la seccion de servicios complementarios </t>
+  </si>
+  <si>
+    <t>1.8.6</t>
+  </si>
+  <si>
+    <t>Se crea la sección "servicios complementarios" trae solamente los ID de Viaje que se activo el servicio complementario.</t>
+  </si>
+  <si>
+    <t>1.8.7</t>
+  </si>
+  <si>
+    <t>En Sidebar de control pagos, se crea 3 sub menus (Flete, Servicios Complementarios y Servicios Aduanales)</t>
   </si>
 </sst>
 </file>
@@ -1851,7 +1899,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36194886-2769-4A79-9B82-6C17CD89E475}">
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="70.77734375" bestFit="1" customWidth="1"/>
@@ -2069,6 +2117,70 @@
       </c>
       <c r="B28" s="4" t="s">
         <v>52</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mejora mostrar el nombre de producto integrado por nombre, calidad y configuracion
</commit_message>
<xml_diff>
--- a/historial de versiones/historial de versiones.xlsx
+++ b/historial de versiones/historial de versiones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ReneGonzalez\nglobal_donpedro\historial de versiones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08113729-0247-4026-BE02-0021DA82B126}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F59C11A2-2E3B-41FE-A916-3085B30CFB3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D8516950-B82A-44A6-A6D8-9588F2ED2E08}"/>
+    <workbookView xWindow="-28908" yWindow="-108" windowWidth="29016" windowHeight="15696" xr2:uid="{D8516950-B82A-44A6-A6D8-9588F2ED2E08}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t>CONTROL DE VERSIONES APP DON PEDRO</t>
   </si>
@@ -247,6 +247,30 @@
   </si>
   <si>
     <t>En Sidebar de control pagos, se crea 3 sub menus (Flete, Servicios Complementarios y Servicios Aduanales)</t>
+  </si>
+  <si>
+    <t>1.8.8</t>
+  </si>
+  <si>
+    <t>Actualizar plantilla de WhatsApp para las alertas, se agrega ID Tracker, Temperatura actual y tiempo de viaje</t>
+  </si>
+  <si>
+    <t>1.8.9</t>
+  </si>
+  <si>
+    <t>Mejora, cuando se le cambia al viaje al estatus "LIBERADO FDA" despues de 20 minutos la app cambia el estatus a "FINALIZADO"</t>
+  </si>
+  <si>
+    <t>1.9.0</t>
+  </si>
+  <si>
+    <t>Mejora, agregar a Archivos Maestros &gt; Productos el campo de temperatura no tolerable</t>
+  </si>
+  <si>
+    <t>1.9.1</t>
+  </si>
+  <si>
+    <t>Mejora, cuando presionen al icono de bote 🗑️ para que inhabilite el producto y no lo elimine</t>
   </si>
 </sst>
 </file>
@@ -284,7 +308,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -294,6 +318,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -310,7 +340,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -327,6 +357,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1899,7 +1932,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36194886-2769-4A79-9B82-6C17CD89E475}">
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="70.77734375" bestFit="1" customWidth="1"/>
@@ -2048,7 +2081,7 @@
       </c>
     </row>
     <row r="20" spans="1:2" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="7" t="s">
         <v>35</v>
       </c>
       <c r="B20" s="4" t="s">
@@ -2181,6 +2214,38 @@
       </c>
       <c r="B36" s="4" t="s">
         <v>68</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>